<commit_message>
Fix missing descriptions when syncing from Supabase.
Backfill description fields from bundled data and add specific KrümCoffee copy for all six locations.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data-source/CeliacSafe_Datenbank_v4_Spain_129_geocoded.xlsx
+++ b/data-source/CeliacSafe_Datenbank_v4_Spain_129_geocoded.xlsx
@@ -36507,17 +36507,17 @@
       <c r="AF86" s="29" t="n"/>
       <c r="AG86" s="29" t="inlineStr">
         <is>
-          <t>Bäckerei/Patisserie in Granollers mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
+          <t>100% glutenfreies KrümCoffee-Café in Granollers mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH86" s="29" t="inlineStr">
         <is>
-          <t>Bakery and patisserie in Granollers offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
+          <t>100% gluten-free KrümCoffee café in Granollers serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI86" s="29" t="inlineStr">
         <is>
-          <t>Panadería y pastelería en Granollers con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
+          <t>Cafetería KrümCoffee 100% sin gluten en Granollers con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ86" s="29" t="n"/>
@@ -36762,17 +36762,17 @@
       <c r="AF87" s="29" t="n"/>
       <c r="AG87" s="29" t="inlineStr">
         <is>
-          <t>Bäckerei/Patisserie in Sant Cugat del Vallès mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
+          <t>100% glutenfreies KrümCoffee-Café in Sant Cugat del Vallès mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH87" s="29" t="inlineStr">
         <is>
-          <t>Bakery and patisserie in Sant Cugat del Vallès offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
+          <t>100% gluten-free KrümCoffee café in Sant Cugat del Vallès serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI87" s="29" t="inlineStr">
         <is>
-          <t>Panadería y pastelería en Sant Cugat del Vallès con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
+          <t>Cafetería KrümCoffee 100% sin gluten en Sant Cugat del Vallès con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ87" s="29" t="n"/>
@@ -37013,17 +37013,17 @@
       <c r="AF88" s="29" t="n"/>
       <c r="AG88" s="29" t="inlineStr">
         <is>
-          <t>Bäckerei/Patisserie in Sabadell mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
+          <t>100% glutenfreies KrümCoffee-Café in Sabadell mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH88" s="29" t="inlineStr">
         <is>
-          <t>Bakery and patisserie in Sabadell offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
+          <t>100% gluten-free KrümCoffee café in Sabadell serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI88" s="29" t="inlineStr">
         <is>
-          <t>Panadería y pastelería en Sabadell con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
+          <t>Cafetería KrümCoffee 100% sin gluten en Sabadell con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ88" s="29" t="n"/>
@@ -37268,17 +37268,17 @@
       <c r="AF89" s="29" t="n"/>
       <c r="AG89" s="29" t="inlineStr">
         <is>
-          <t>Bäckerei/Patisserie in Olesa de Montserrat mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
+          <t>100% glutenfreies KrümCoffee-Café in Olesa de Montserrat mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH89" s="29" t="inlineStr">
         <is>
-          <t>Bakery and patisserie in Olesa de Montserrat offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
+          <t>100% gluten-free KrümCoffee café in Olesa de Montserrat serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI89" s="29" t="inlineStr">
         <is>
-          <t>Panadería y pastelería en Olesa de Montserrat con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
+          <t>Cafetería KrümCoffee 100% sin gluten en Olesa de Montserrat con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ89" s="29" t="n"/>
@@ -37523,17 +37523,17 @@
       <c r="AF90" s="29" t="n"/>
       <c r="AG90" s="29" t="inlineStr">
         <is>
-          <t>Bäckerei/Patisserie in Vic mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
+          <t>100% glutenfreies KrümCoffee-Café in Vic mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH90" s="29" t="inlineStr">
         <is>
-          <t>Bakery and patisserie in Vic offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
+          <t>100% gluten-free KrümCoffee café in Vic serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI90" s="29" t="inlineStr">
         <is>
-          <t>Panadería y pastelería en Vic con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
+          <t>Cafetería KrümCoffee 100% sin gluten en Vic con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ90" s="29" t="n"/>
@@ -37778,17 +37778,17 @@
       <c r="AF91" s="29" t="n"/>
       <c r="AG91" s="29" t="inlineStr">
         <is>
-          <t>Bäckerei/Patisserie in Jerez de la Frontera mit Brot, Brötchen, Kuchen, Torten, Gebäck, süßen Backwaren und teilweise herzhaften Snacks.</t>
+          <t>100% glutenfreies KrümCoffee-Café in Jerez de la Frontera mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH91" s="29" t="inlineStr">
         <is>
-          <t>Bakery and patisserie in Jerez de la Frontera offering bread, rolls, cakes, tarts, pastries, sweet baked goods, and a selection of savoury snacks.</t>
+          <t>100% gluten-free KrümCoffee café in Jerez de la Frontera serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI91" s="29" t="inlineStr">
         <is>
-          <t>Panadería y pastelería en Jerez de la Frontera con pan, panecillos, tartas, pasteles, bollería, dulces y algunos snacks salados.</t>
+          <t>Cafetería KrümCoffee 100% sin gluten en Jerez de la Frontera con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ91" s="29" t="n"/>

</xml_diff>

<commit_message>
Add profile dietary filters, map pin UX, and food-focused restaurant descriptions.
Profile switches for lactose-free, vegan, and wheat-free preferences persist locally and filter search and map results. Map pins use category colors with a bottom preview card. Restaurant descriptions drop audit-style copy in favor of dish-focused text across Excel, JSON, and normalization scripts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data-source/CeliacSafe_Datenbank_v4_Spain_129_geocoded.xlsx
+++ b/data-source/CeliacSafe_Datenbank_v4_Spain_129_geocoded.xlsx
@@ -36507,17 +36507,17 @@
       <c r="AF86" s="29" t="n"/>
       <c r="AG86" s="29" t="inlineStr">
         <is>
-          <t>100% glutenfreies KrümCoffee-Café in Granollers mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
+          <t>KrümCoffee-Café in Granollers mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH86" s="29" t="inlineStr">
         <is>
-          <t>100% gluten-free KrümCoffee café in Granollers serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
+          <t>KrümCoffee café in Granollers serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI86" s="29" t="inlineStr">
         <is>
-          <t>Cafetería KrümCoffee 100% sin gluten en Granollers con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
+          <t>Cafetería KrümCoffee en Granollers con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ86" s="29" t="n"/>
@@ -36762,17 +36762,17 @@
       <c r="AF87" s="29" t="n"/>
       <c r="AG87" s="29" t="inlineStr">
         <is>
-          <t>100% glutenfreies KrümCoffee-Café in Sant Cugat del Vallès mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
+          <t>KrümCoffee-Café in Sant Cugat del Vallès mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH87" s="29" t="inlineStr">
         <is>
-          <t>100% gluten-free KrümCoffee café in Sant Cugat del Vallès serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
+          <t>KrümCoffee café in Sant Cugat del Vallès serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI87" s="29" t="inlineStr">
         <is>
-          <t>Cafetería KrümCoffee 100% sin gluten en Sant Cugat del Vallès con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
+          <t>Cafetería KrümCoffee en Sant Cugat del Vallès con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ87" s="29" t="n"/>
@@ -37013,17 +37013,17 @@
       <c r="AF88" s="29" t="n"/>
       <c r="AG88" s="29" t="inlineStr">
         <is>
-          <t>100% glutenfreies KrümCoffee-Café in Sabadell mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
+          <t>KrümCoffee-Café in Sabadell mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH88" s="29" t="inlineStr">
         <is>
-          <t>100% gluten-free KrümCoffee café in Sabadell serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
+          <t>KrümCoffee café in Sabadell serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI88" s="29" t="inlineStr">
         <is>
-          <t>Cafetería KrümCoffee 100% sin gluten en Sabadell con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
+          <t>Cafetería KrümCoffee en Sabadell con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ88" s="29" t="n"/>
@@ -37268,17 +37268,17 @@
       <c r="AF89" s="29" t="n"/>
       <c r="AG89" s="29" t="inlineStr">
         <is>
-          <t>100% glutenfreies KrümCoffee-Café in Olesa de Montserrat mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
+          <t>KrümCoffee-Café in Olesa de Montserrat mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH89" s="29" t="inlineStr">
         <is>
-          <t>100% gluten-free KrümCoffee café in Olesa de Montserrat serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
+          <t>KrümCoffee café in Olesa de Montserrat serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI89" s="29" t="inlineStr">
         <is>
-          <t>Cafetería KrümCoffee 100% sin gluten en Olesa de Montserrat con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
+          <t>Cafetería KrümCoffee en Olesa de Montserrat con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ89" s="29" t="n"/>
@@ -37523,17 +37523,17 @@
       <c r="AF90" s="29" t="n"/>
       <c r="AG90" s="29" t="inlineStr">
         <is>
-          <t>100% glutenfreies KrümCoffee-Café in Vic mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
+          <t>KrümCoffee-Café in Vic mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH90" s="29" t="inlineStr">
         <is>
-          <t>100% gluten-free KrümCoffee café in Vic serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
+          <t>KrümCoffee café in Vic serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI90" s="29" t="inlineStr">
         <is>
-          <t>Cafetería KrümCoffee 100% sin gluten en Vic con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
+          <t>Cafetería KrümCoffee en Vic con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ90" s="29" t="n"/>
@@ -37778,17 +37778,17 @@
       <c r="AF91" s="29" t="n"/>
       <c r="AG91" s="29" t="inlineStr">
         <is>
-          <t>100% glutenfreies KrümCoffee-Café in Jerez de la Frontera mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
+          <t>KrümCoffee-Café in Jerez de la Frontera mit Kaffee, Frühstück, Brunch, Kuchen, Gebäck und herzhaften Snacks.</t>
         </is>
       </c>
       <c r="AH91" s="29" t="inlineStr">
         <is>
-          <t>100% gluten-free KrümCoffee café in Jerez de la Frontera serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
+          <t>KrümCoffee café in Jerez de la Frontera serving coffee, breakfast, brunch, cakes, pastries, and savoury snacks.</t>
         </is>
       </c>
       <c r="AI91" s="29" t="inlineStr">
         <is>
-          <t>Cafetería KrümCoffee 100% sin gluten en Jerez de la Frontera con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
+          <t>Cafetería KrümCoffee en Jerez de la Frontera con café, desayuno, brunch, tartas, bollería y snacks salados.</t>
         </is>
       </c>
       <c r="AJ91" s="29" t="n"/>

</xml_diff>